<commit_message>
Harden reasoning-model pilot settings
</commit_message>
<xml_diff>
--- a/workbooks/TurkCuisineBench_Pilot_Execution_v0.3_configured.xlsx
+++ b/workbooks/TurkCuisineBench_Pilot_Execution_v0.3_configured.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfab0e1bebf4d4dce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Settings" sheetId="2" r:id="R96e1c1c7ce2e41be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Items" sheetId="3" r:id="Rc5c4aa72a59a487c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requests" sheetId="4" r:id="R4b3789e9beb34e98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Responses" sheetId="5" r:id="R267c52b373cc4483"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalization_Tests" sheetId="6" r:id="R26653c3ba26743e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="7" r:id="R6f9a54c2e01e474f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Freeze_Record" sheetId="8" r:id="R648865f93dbf476a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd3d8394c565b48fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Settings" sheetId="2" r:id="R6ec50e5e29d14308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Items" sheetId="3" r:id="Rc05ae9db06cf40de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requests" sheetId="4" r:id="Re2de30e422ac491f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Responses" sheetId="5" r:id="Rcdf9c903a3f548fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalization_Tests" sheetId="6" r:id="Rdc8e4fe28ce545ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="7" r:id="Rbcd39e71bb534216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Freeze_Record" sheetId="8" r:id="R25e3bca7a7264b0d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -969,7 +969,7 @@
         <x:v>Maximum output</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>64 tokens</x:v>
+        <x:v>256 tokens</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1022,9 +1022,17 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="20" t="str">
+        <x:v>Reasoning effort</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="str">
+        <x:v>low (both models)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
         <x:v>Secrets</x:v>
       </x:c>
-      <x:c r="B18" s="14" t="str">
+      <x:c r="B19" t="str">
         <x:v>Environment variables only</x:v>
       </x:c>
     </x:row>
@@ -3115,7 +3123,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcfa67a9edaf4fc2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc77cf60c15994d4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5208,7 +5216,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebb2a094bdd44fec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0245be66cd4f40ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8442,7 +8450,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80418c5bb5084e4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc50b4e345d35467c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8665,7 +8673,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96d0d57cb10d4900"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a07a4cfab5d450d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>